<commit_message>
genration de bulletin de semestriel secondaire
</commit_message>
<xml_diff>
--- a/public/models/Matieres.xlsx
+++ b/public/models/Matieres.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29530"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBE96D61-C780-4F92-BEB4-C3D4110413E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -14,15 +15,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
     <t>Nom</t>
   </si>
+  <si>
+    <t>Type de matière</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -72,9 +76,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -112,9 +116,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -149,7 +153,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -184,7 +188,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -357,13 +361,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>